<commit_message>
Add new test cases
</commit_message>
<xml_diff>
--- a/G1_Acceptance.Ass1.xlsx
+++ b/G1_Acceptance.Ass1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\almo1\GoNature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\reutd\GoNature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0673A816-B5C5-4248-8DD8-DE2382FF91CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322FDECC-3AFE-4714-926F-BB0E86C10215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="1" xr2:uid="{66F18C86-3E6B-4F2E-A3A6-956843228F2B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{66F18C86-3E6B-4F2E-A3A6-956843228F2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="256">
   <si>
     <t>Req. number</t>
   </si>
@@ -610,12 +610,414 @@
   <si>
     <t>Checking that a guide can enter waiting line.</t>
   </si>
+  <si>
+    <t>ChangeCapacityRequestGapSuccessful</t>
+  </si>
+  <si>
+    <t>Park manager presses "change capacity"
+chooses park: "Banias Nature Reserve"
+sets capacity= "200"
+presses "Send request"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A request is sent for the department manager's approval and the message "Request Sent" is displayed
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The manager is registered as the park manager and the parks capacity is already defined </t>
+  </si>
+  <si>
+    <t>Successful capacity change request</t>
+  </si>
+  <si>
+    <t>ChangeCapacityRequestUnSuccessfulNegative</t>
+  </si>
+  <si>
+    <t>Park manager presses "change capacity"
+chooses park: "Banias Nature Reserve"
+set capacity= "-200"
+presses "Send request"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The system will not send a request to the department manager and the message "Invalid capacity" is displayed
+</t>
+  </si>
+  <si>
+    <t>UnSuccessful capacity change request (negative)</t>
+  </si>
+  <si>
+    <t>ConfirmCapacityChangeSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Department manager presses "Capacity change requests" and selects a request from the list, 
+the request opens:
+park: Banias Nature Reserve
+requested capacity: 200
+current capacity: 300 
+ manager presses "confirm request"
+   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banias Nature Reserve capacity changed to 200 and the message "Request confirmed" is displayed
+</t>
+  </si>
+  <si>
+    <t>The manager is registered as the department manager and a capacity change request was sent</t>
+  </si>
+  <si>
+    <t>Successful capacity change request confrmation</t>
+  </si>
+  <si>
+    <t>RejectCapacityChangeSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Department manager presses "Capacity change requests" and selects a request from the list, 
+the request opens:
+park: Banias Nature Reserve
+requested capacity: 200
+current capacity: 300 
+ manager presses "reject request"
+   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banias Nature Reserve capacity remains to 300 and the message "Request rejected" is displayed
+</t>
+  </si>
+  <si>
+    <t>Successful capacity change request rejection</t>
+  </si>
+  <si>
+    <t>DefineQuotaCapacityGapRequestSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Park manager presses "define wanted capacity-qouta gap". 
+chooses park: "Banias Nature Reserve"
+The park's capacity= 200 
+Manager defines the gap to be 50   </t>
+  </si>
+  <si>
+    <t>A request is sent for the department manager's approval and the message "Request Sent" is displayed</t>
+  </si>
+  <si>
+    <t>Successful gap definition request</t>
+  </si>
+  <si>
+    <t>DefineQuotaCapacityGapUnSuccessfulNegative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Park manager presses "define wanted capacity-qouta gap".
+chooses park: "Banias Nature Reserve" 
+The park's capacity= 200 
+Manager defines the gap to be -50
+presses "Send request"   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The system will not send a request to the department manager and the message "Invalid gap value" is displayed
+</t>
+  </si>
+  <si>
+    <t>UnSuccessful gap definition request (negative gap)</t>
+  </si>
+  <si>
+    <t>DefineQuotaCapacityGapUnSuccessfulLargerThanCapacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Park manager presses "define wanted capacity-qouta gap".
+chooses park: "Banias Nature Reserve" 
+The park's capacity= 200 
+Manager defines the gap= 250
+presses "Send request"   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The manager is registered as the park manager and the parks capacity and quota - capacity gap are already defined </t>
+  </si>
+  <si>
+    <t>UnSuccessful gap definition request (gap bigger than the defined capacity)</t>
+  </si>
+  <si>
+    <t>ConfirmGapDefinitionSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Department manager presses "Quota - capacity gap definition requests" and selects a request from the list, 
+the request opens:
+park: Banias Nature Reserve
+requested gap: 200  
+manager presses "confirm request"
+   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banias Nature Reserve quota - capacity gap defined to 200 and the message "Request confirmed" is displayed
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The manager is registered as the department manager and a quota- capacity gap definition request was sent  </t>
+  </si>
+  <si>
+    <t>Successful gap definition request confirmation</t>
+  </si>
+  <si>
+    <t>RejectGapDefinitionSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Department manager presses "Quota - capacity gap definition requests" and selects a request from the list, 
+the request opens:
+park: Banias Nature Reserve
+requested gap: 200  
+manager presses "reject request"
+   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banias Nature Reserve quota - capacity gap remains undefined and the message "Request rejected" is displayed
+</t>
+  </si>
+  <si>
+    <t>Successful gap definition request rejection</t>
+  </si>
+  <si>
+    <t>ChangeQuotaCapacityGapSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Park manager presses "define wanted capacity-qouta gap".
+chooses park: "Banias Nature Reserve" 
+The park's capacity= 200
+ Manager sets the gap to 50 
+presses "Send request"  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The system will not send a request to the department manager and the message "Invalid gap value" is displayed 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The manager is registered as the park manager and the parks capacity and gap are already defined </t>
+  </si>
+  <si>
+    <t>Successful gap change request</t>
+  </si>
+  <si>
+    <t>ChangeQuotaCapacityGapUnSuccessfulNegative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Park manager signs in and presses "change capacity-qouta gap".
+chooses park: "Banias Nature Reserve" 
+The park's capacity= 200 
+Manager changes the gap = -50
+presses "Send request"   </t>
+  </si>
+  <si>
+    <t>UnSuccessful gap change request (negative gap)</t>
+  </si>
+  <si>
+    <t>ChangeQuotaCapacityGapUnSuccessfulLargerThanCapacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Park manager signs in and presses "change capacity-qouta gap".
+chooses park: "Banias Nature Reserve" 
+The park's capacity= 200 
+Manager defines the gap to 250   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The system will not confirm the change
+</t>
+  </si>
+  <si>
+    <t>UnSuccessful gap change request (gap bigger than the defined capacity)</t>
+  </si>
+  <si>
+    <t>ConfirmGapChangeSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Department manager signs in and presses "Quota - capacity  gap change requests" and selects a request from the list, 
+the request opens:
+park: Banias Nature Reserve
+requested gap: 200
+current gap: 300 
+manager presses "confirm request"
+   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banias Nature Reserve quota - capacity gap changed to 200 and the message "Request confirmed" is displayed
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The manager is registered as the department manager and a quota- capacity gap change request was sent  </t>
+  </si>
+  <si>
+    <t>Successful gap change request confirmation</t>
+  </si>
+  <si>
+    <t>RejectGapChangeSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Department manager signs in and presses "Quota - capacity  gap change requests" and selects a request from the list, 
+the request opens:
+park: Banias Nature Reserve
+requested gap: 200
+current gap: 300 
+manager presses "reject request"
+   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banias Nature Reserve quota - capacity gap remains 300 and the message "Request rejectod" is displayed
+</t>
+  </si>
+  <si>
+    <t>Successful gap change request rejection</t>
+  </si>
+  <si>
+    <t>AvgStayTimeCalculation</t>
+  </si>
+  <si>
+    <t>????????????</t>
+  </si>
+  <si>
+    <t>ChangeEstimatedStayTimeRequestSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Park manager presses "change estimated stay time ".
+chooses park: "Banias Nature Reserve" 
+current stay time: 2.5 hours
+wanted stay time: 3 hours
+presses "Send reqest"   </t>
+  </si>
+  <si>
+    <t>The manager is registered as the park manager</t>
+  </si>
+  <si>
+    <t>Successful estimated stay time change request</t>
+  </si>
+  <si>
+    <t>ChangeEstimatedStayTimeRequestUnSuccessfulNegative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Park manager presses "change estimated stay time ".
+chooses park: "Banias Nature Reserve" 
+current stay time: 2.5 hours
+wanted stay time: -3 hours
+presses "Send reqest"   </t>
+  </si>
+  <si>
+    <t>The system will not send a request to the department manager and the message "Invalid stay time" is displayed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unsuccessful estimated stay time change request (negative) </t>
+  </si>
+  <si>
+    <t>ConfirmEstimatedStayTimeChangeSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Department manager presses "estimated stay time change requests" and selects a request from the list, 
+the request opens:
+park: Banias Nature Reserve
+requested stay time: 3   
+manager presses "confirm request"
+   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banias Nature Reserve estimated stay time changes to 3 hours and the message "Request confirmed" is displayed
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The manager is registered as the department manager and an estimated stay time change request was sent  </t>
+  </si>
+  <si>
+    <t>Successful estimated stay time change approval</t>
+  </si>
+  <si>
+    <t>RejectEstimatedStayTimeChangeSuccessful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Department manager presses "estimated stay time change requests" and selects a request from the list, 
+the request opens:
+park: Banias Nature Reserve
+requested stay time: 3   
+manager presses "reject request"
+   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banias Nature Reserve estimated stay time doesn’t change and the message "Request rejected" is displayed
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BookingCancled_SeeReservationTable </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open booking screen
+Enter visitor ID
+Select park: Banias Nature Reserve
+Select date and time: 15/04/2026 10:00
+Enter number of visitors: 3
+Enter e-mail: visitor@gmail.com
+Click "book visit" button
+Choose "Reservation Table"  
+</t>
+  </si>
+  <si>
+    <t>The system informs the user that no space is available for selected visit time.
+The system does not create a reservation.
+The system allows the user to see the resrvation table in order to choose another date or join the waiting list.</t>
+  </si>
+  <si>
+    <t>The system is on the booking screen.
+Banias Nature Reserve has no available capacity for 3 visitors on 15/04/2026 at 10:00.
+Banias Nature Reserve's capacity: 1000
+Qouta- capacity gap: 200
+There are already 800 spots booked for the mentioned time at the park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bookings quota reached, reseration cancle, users chooses to look at the reservations table </t>
+  </si>
+  <si>
+    <t>OrdererAprrovesReminder</t>
+  </si>
+  <si>
+    <t>Orderer "Israel Israeli" receives an 
+e-mail and SMS saying "Dear Israel Israeli, please approve your visit in Banias Nature Reserve tommorow at 2pm within the next 2 hours by pressing the link below….".
+Israel immediately sees and approves his visit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The system accepts the approval and won't aoutmatically cancel the reservation </t>
+  </si>
+  <si>
+    <t>The user's reservation exists in the system with the correct e-mail address and phone number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">user receives a reminder to their visit tommorow and doesn't approve it before aoutomtic cancellation  </t>
+  </si>
+  <si>
+    <t>OrdererMissesReminderAutoCancel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orderer "Israel Israeli" receives an 
+e-mail and SMS saying "Dear Israel Israeli, please approve your visit in Banias Nature Reserve tommorow at 2pm within the next 2 hours by pressing the link below….".
+Israel sees message 3 hours too late, and can't approve his visit  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The system aoutmatically cancels the reservation two hours after he message was sent </t>
+  </si>
+  <si>
+    <t xml:space="preserve">user receives a reminder to their visit tommorow and approves it before aoutomtic cancellation  </t>
+  </si>
+  <si>
+    <t>AutoCancelMessage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A reservation was automatically canceled </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The system sents the orderer a cancellation message by e-mail and SMS saying "Dear Traveler, due to reminder disapproval, we had to cancel your visit tommorow."  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A reminder for a reservation wasn't approved in time </t>
+  </si>
+  <si>
+    <t xml:space="preserve">automtic cancellation message sent   </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -673,6 +1075,21 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -688,7 +1105,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -711,11 +1128,71 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -743,6 +1220,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1065,14 +1557,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABE2F884-F2EF-4287-AC3D-5537D5275C3C}">
   <dimension ref="A1:C82"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5" customWidth="1"/>
-    <col min="2" max="2" width="88.125" customWidth="1"/>
-    <col min="3" max="3" width="5.25" customWidth="1"/>
+    <col min="2" max="2" width="88.09765625" customWidth="1"/>
+    <col min="3" max="3" width="5.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="105.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1083,7 +1575,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1094,7 +1586,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1105,7 +1597,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1116,7 +1608,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1127,7 +1619,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1138,7 +1630,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1149,7 +1641,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1160,7 +1652,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1171,7 +1663,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1182,7 +1674,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1193,7 +1685,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1204,7 +1696,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1215,7 +1707,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1226,7 +1718,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1237,7 +1729,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1248,7 +1740,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -1259,7 +1751,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1270,7 +1762,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1281,7 +1773,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1292,7 +1784,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1303,7 +1795,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1314,7 +1806,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1325,7 +1817,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1336,7 +1828,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1347,7 +1839,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1358,7 +1850,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1369,7 +1861,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1380,7 +1872,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1391,7 +1883,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1402,7 +1894,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1413,7 +1905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1424,7 +1916,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1435,7 +1927,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1446,7 +1938,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1457,7 +1949,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1468,7 +1960,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1479,7 +1971,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1490,7 +1982,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1501,7 +1993,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1512,7 +2004,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1523,7 +2015,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1534,7 +2026,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1545,7 +2037,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1556,7 +2048,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1567,7 +2059,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1578,7 +2070,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1589,7 +2081,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1600,7 +2092,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1611,7 +2103,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1622,7 +2114,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1633,7 +2125,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1644,7 +2136,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1655,7 +2147,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1666,7 +2158,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1677,7 +2169,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1688,7 +2180,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1699,7 +2191,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1710,7 +2202,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1721,7 +2213,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1732,7 +2224,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -1743,7 +2235,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -1754,7 +2246,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -1765,7 +2257,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -1776,7 +2268,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -1787,7 +2279,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -1798,7 +2290,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -1809,7 +2301,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -1820,7 +2312,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -1831,7 +2323,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -1842,7 +2334,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -1853,7 +2345,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -1864,7 +2356,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -1875,7 +2367,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -1886,7 +2378,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>74</v>
       </c>
@@ -1897,7 +2389,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>75</v>
       </c>
@@ -1908,7 +2400,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>76</v>
       </c>
@@ -1919,7 +2411,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>77</v>
       </c>
@@ -1930,7 +2422,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>78</v>
       </c>
@@ -1941,7 +2433,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>79</v>
       </c>
@@ -1952,7 +2444,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>80</v>
       </c>
@@ -1971,17 +2463,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A028A801-0122-4DDE-8D73-57AF100E1B01}">
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Z41"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="79.75" customWidth="1"/>
-    <col min="2" max="2" width="27.75" customWidth="1"/>
-    <col min="3" max="3" width="39.25" customWidth="1"/>
-    <col min="4" max="4" width="24.75" customWidth="1"/>
+    <col min="1" max="1" width="79.69921875" customWidth="1"/>
+    <col min="2" max="2" width="27.69921875" customWidth="1"/>
+    <col min="3" max="3" width="39.19921875" customWidth="1"/>
+    <col min="4" max="4" width="24.69921875" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1998,7 +2490,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" s="2" customFormat="1" ht="55.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>90</v>
       </c>
@@ -2015,7 +2507,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="6" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" s="6" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>95</v>
       </c>
@@ -2032,7 +2524,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="100.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="83.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>100</v>
       </c>
@@ -2049,7 +2541,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="86.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="83.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>105</v>
       </c>
@@ -2066,7 +2558,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="100.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="97.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>107</v>
       </c>
@@ -2083,7 +2575,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="57.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="55.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>109</v>
       </c>
@@ -2100,7 +2592,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="129" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="124.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>114</v>
       </c>
@@ -2117,7 +2609,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="129" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="124.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
         <v>119</v>
       </c>
@@ -2134,7 +2626,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="129" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="124.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>121</v>
       </c>
@@ -2151,7 +2643,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="129" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="124.8" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>126</v>
       </c>
@@ -2168,7 +2660,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="143.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="138.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>131</v>
       </c>
@@ -2185,7 +2677,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="72" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>136</v>
       </c>
@@ -2202,7 +2694,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="72" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
         <v>141</v>
       </c>
@@ -2219,7 +2711,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="86.25" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="83.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>145</v>
       </c>
@@ -2236,7 +2728,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="214.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="207.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>150</v>
       </c>
@@ -2253,7 +2745,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="214.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="207.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
         <v>155</v>
       </c>
@@ -2269,6 +2761,492 @@
       <c r="E17" s="9" t="s">
         <v>158</v>
       </c>
+    </row>
+    <row r="18" spans="1:5" ht="88.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="90.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="157.80000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="157.80000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="135.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="135.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="135.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
+        <v>210</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="57.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+    </row>
+    <row r="33" spans="1:26" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="34" spans="1:26" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="35" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="36" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>235</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="37" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>235</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="38" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="15"/>
+      <c r="K38" s="15"/>
+      <c r="L38" s="15"/>
+      <c r="M38" s="15"/>
+      <c r="N38" s="15"/>
+      <c r="O38" s="15"/>
+      <c r="P38" s="15"/>
+      <c r="Q38" s="15"/>
+      <c r="R38" s="15"/>
+      <c r="S38" s="15"/>
+      <c r="T38" s="15"/>
+      <c r="U38" s="15"/>
+      <c r="V38" s="15"/>
+      <c r="W38" s="15"/>
+      <c r="X38" s="15"/>
+      <c r="Y38" s="15"/>
+      <c r="Z38" s="15"/>
+    </row>
+    <row r="39" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="13" t="s">
+        <v>242</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="E39" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="15"/>
+      <c r="I39" s="15"/>
+      <c r="J39" s="15"/>
+      <c r="K39" s="15"/>
+      <c r="L39" s="15"/>
+      <c r="M39" s="15"/>
+      <c r="N39" s="15"/>
+      <c r="O39" s="15"/>
+      <c r="P39" s="15"/>
+      <c r="Q39" s="15"/>
+      <c r="R39" s="15"/>
+      <c r="S39" s="15"/>
+      <c r="T39" s="15"/>
+      <c r="U39" s="15"/>
+      <c r="V39" s="15"/>
+      <c r="W39" s="15"/>
+      <c r="X39" s="15"/>
+      <c r="Y39" s="15"/>
+      <c r="Z39" s="15"/>
+    </row>
+    <row r="40" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="E40" s="14" t="s">
+        <v>250</v>
+      </c>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15"/>
+      <c r="K40" s="15"/>
+      <c r="L40" s="15"/>
+      <c r="M40" s="15"/>
+      <c r="N40" s="15"/>
+      <c r="O40" s="15"/>
+      <c r="P40" s="15"/>
+      <c r="Q40" s="15"/>
+      <c r="R40" s="15"/>
+      <c r="S40" s="15"/>
+      <c r="T40" s="15"/>
+      <c r="U40" s="15"/>
+      <c r="V40" s="15"/>
+      <c r="W40" s="15"/>
+      <c r="X40" s="15"/>
+      <c r="Y40" s="15"/>
+      <c r="Z40" s="15"/>
+    </row>
+    <row r="41" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>252</v>
+      </c>
+      <c r="C41" s="14" t="s">
+        <v>253</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
+      <c r="I41" s="15"/>
+      <c r="J41" s="15"/>
+      <c r="K41" s="15"/>
+      <c r="L41" s="15"/>
+      <c r="M41" s="15"/>
+      <c r="N41" s="15"/>
+      <c r="O41" s="15"/>
+      <c r="P41" s="15"/>
+      <c r="Q41" s="15"/>
+      <c r="R41" s="15"/>
+      <c r="S41" s="15"/>
+      <c r="T41" s="15"/>
+      <c r="U41" s="15"/>
+      <c r="V41" s="15"/>
+      <c r="W41" s="15"/>
+      <c r="X41" s="15"/>
+      <c r="Y41" s="15"/>
+      <c r="Z41" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2279,16 +3257,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F57B142-739C-42E7-8832-36341E864322}">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="55.25" customWidth="1"/>
-    <col min="2" max="2" width="32.625" customWidth="1"/>
-    <col min="3" max="3" width="51.625" customWidth="1"/>
-    <col min="4" max="4" width="34.625" customWidth="1"/>
+    <col min="1" max="1" width="55.19921875" customWidth="1"/>
+    <col min="2" max="2" width="32.59765625" customWidth="1"/>
+    <col min="3" max="3" width="51.59765625" customWidth="1"/>
+    <col min="4" max="4" width="34.59765625" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -2305,92 +3283,92 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" ht="83.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" s="2" customFormat="1" ht="83.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="83.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" s="2" customFormat="1" ht="83.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" spans="1:5" s="2" customFormat="1" ht="83.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" s="2" customFormat="1" ht="83.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
     </row>
-    <row r="5" spans="1:5" s="2" customFormat="1" ht="83.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" s="2" customFormat="1" ht="83.85" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
-    <row r="6" spans="1:5" s="6" customFormat="1" ht="84.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" s="6" customFormat="1" ht="84.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
-    <row r="7" spans="1:5" s="6" customFormat="1" ht="81" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" s="6" customFormat="1" ht="81" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
-    <row r="8" spans="1:5" s="6" customFormat="1" ht="71.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" s="6" customFormat="1" ht="71.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
-    <row r="9" spans="1:5" s="6" customFormat="1" ht="71.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" s="6" customFormat="1" ht="71.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:5" s="6" customFormat="1" ht="71.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" s="6" customFormat="1" ht="71.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" spans="1:5" ht="79.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="79.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" spans="1:5" ht="73.150000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="73.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
     </row>
-    <row r="13" spans="1:5" ht="78.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="78.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="5"/>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" spans="1:5" ht="42.4" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="15" spans="1:5" ht="76.900000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="42.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:5" ht="76.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C16" s="5"/>
     </row>
   </sheetData>
@@ -2402,7 +3380,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD60C334-447E-4123-A1B5-2C4F489DB128}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add a new test case
</commit_message>
<xml_diff>
--- a/G1_Acceptance.Ass1.xlsx
+++ b/G1_Acceptance.Ass1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\reutd\GoNature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{322FDECC-3AFE-4714-926F-BB0E86C10215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE5C69C1-929D-449B-ABE2-7CF698134464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{66F18C86-3E6B-4F2E-A3A6-956843228F2B}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="259">
   <si>
     <t>Req. number</t>
   </si>
@@ -867,9 +867,6 @@
     <t>AvgStayTimeCalculation</t>
   </si>
   <si>
-    <t>????????????</t>
-  </si>
-  <si>
     <t>ChangeEstimatedStayTimeRequestSuccessful</t>
   </si>
   <si>
@@ -1011,6 +1008,23 @@
   </si>
   <si>
     <t xml:space="preserve">automtic cancellation message sent   </t>
+  </si>
+  <si>
+    <t>Average Stay Time Calculation for Park Visitors</t>
+  </si>
+  <si>
+    <t>Enter the park visit history screen.
+Choose the following visits:
+1. A group of 5 people spent 2 hours at the park
+2. 1 person spent 8 hours at the park
+Press "Calculate average stay time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The message "Average stay time calculated: 3 hours" will appear  on the screen </t>
+  </si>
+  <si>
+    <t xml:space="preserve">A park exists in the system
+A few visits are recorded in the system (number of people and stay time for each reservation) </t>
   </si>
 </sst>
 </file>
@@ -1105,7 +1119,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1188,11 +1202,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1235,6 +1260,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2467,7 +2495,7 @@
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="79.69921875" customWidth="1"/>
-    <col min="2" max="2" width="27.69921875" customWidth="1"/>
+    <col min="2" max="2" width="36.8984375" customWidth="1"/>
     <col min="3" max="3" width="39.19921875" customWidth="1"/>
     <col min="4" max="4" width="24.69921875" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
@@ -2983,7 +3011,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="136.80000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
         <v>215</v>
       </c>
@@ -3000,117 +3028,123 @@
         <v>218</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="57.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" ht="131.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="B32" s="12" t="s">
-        <v>220</v>
-      </c>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
+      <c r="B32" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="33" spans="1:26" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="B33" s="12" t="s">
         <v>221</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>222</v>
       </c>
       <c r="C33" s="12" t="s">
         <v>179</v>
       </c>
       <c r="D33" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="E33" s="12" t="s">
         <v>223</v>
-      </c>
-      <c r="E33" s="12" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="34" spans="1:26" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="B34" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="B34" s="12" t="s">
+      <c r="C34" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="D34" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="E34" s="12" t="s">
         <v>227</v>
-      </c>
-      <c r="D34" s="12" t="s">
-        <v>223</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="35" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="C35" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="D35" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="D35" s="12" t="s">
+      <c r="E35" s="12" t="s">
         <v>232</v>
-      </c>
-      <c r="E35" s="12" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="36" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="B36" s="12" t="s">
         <v>234</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="C36" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C36" s="12" t="s">
-        <v>236</v>
-      </c>
       <c r="D36" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="E36" s="12" t="s">
         <v>232</v>
-      </c>
-      <c r="E36" s="12" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="37" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="B37" s="12" t="s">
         <v>234</v>
       </c>
-      <c r="B37" s="12" t="s">
+      <c r="C37" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C37" s="12" t="s">
-        <v>236</v>
-      </c>
       <c r="D37" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="E37" s="12" t="s">
         <v>232</v>
-      </c>
-      <c r="E37" s="12" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="38" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="B38" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="B38" s="14" t="s">
+      <c r="C38" s="14" t="s">
         <v>238</v>
       </c>
-      <c r="C38" s="14" t="s">
+      <c r="D38" s="14" t="s">
         <v>239</v>
       </c>
-      <c r="D38" s="14" t="s">
+      <c r="E38" s="14" t="s">
         <v>240</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>241</v>
       </c>
       <c r="F38" s="15"/>
       <c r="G38" s="15"/>
@@ -3136,19 +3170,19 @@
     </row>
     <row r="39" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="B39" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="B39" s="14" t="s">
+      <c r="C39" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="C39" s="14" t="s">
+      <c r="D39" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="D39" s="14" t="s">
+      <c r="E39" s="14" t="s">
         <v>245</v>
-      </c>
-      <c r="E39" s="14" t="s">
-        <v>246</v>
       </c>
       <c r="F39" s="15"/>
       <c r="G39" s="15"/>
@@ -3174,19 +3208,19 @@
     </row>
     <row r="40" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="B40" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="C40" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="C40" s="14" t="s">
+      <c r="D40" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="E40" s="14" t="s">
         <v>249</v>
-      </c>
-      <c r="D40" s="14" t="s">
-        <v>245</v>
-      </c>
-      <c r="E40" s="14" t="s">
-        <v>250</v>
       </c>
       <c r="F40" s="15"/>
       <c r="G40" s="15"/>
@@ -3212,19 +3246,19 @@
     </row>
     <row r="41" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="B41" s="14" t="s">
         <v>251</v>
       </c>
-      <c r="B41" s="14" t="s">
+      <c r="C41" s="14" t="s">
         <v>252</v>
       </c>
-      <c r="C41" s="14" t="s">
+      <c r="D41" s="14" t="s">
         <v>253</v>
       </c>
-      <c r="D41" s="14" t="s">
+      <c r="E41" s="14" t="s">
         <v>254</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>255</v>
       </c>
       <c r="F41" s="15"/>
       <c r="G41" s="15"/>

</xml_diff>

<commit_message>
Update excel file, gal's tests
</commit_message>
<xml_diff>
--- a/G1_Acceptance.Ass1.xlsx
+++ b/G1_Acceptance.Ass1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\reutd\GoNature\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rygra\GoNature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BC66BB9-75FB-4E80-9ACE-AC56652F95A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53314E48-F03D-4BD4-9D93-D158BE75C2DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{66F18C86-3E6B-4F2E-A3A6-956843228F2B}"/>
+    <workbookView xWindow="1170" yWindow="495" windowWidth="22950" windowHeight="15705" activeTab="1" xr2:uid="{66F18C86-3E6B-4F2E-A3A6-956843228F2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="344">
   <si>
     <t>Req. number</t>
   </si>
@@ -1032,16 +1032,424 @@
 Reut Dahan, reut.dahan@e.braude.ac.il
 date: </t>
   </si>
+  <si>
+    <t>CheckAvailableSpots_HasSpace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open "Availability" screen
+Select park : Banias Nature Reserve
+Select date &amp; time : 07/04/2026, 10:00
+</t>
+  </si>
+  <si>
+    <t>The system displays the exact number of available spots
+(e.g. "50 available spots")</t>
+  </si>
+  <si>
+    <t>Banias Nature Reserve has 50 available spots for 07/04/2026 at 10:00</t>
+  </si>
+  <si>
+    <t>checking that the system displays available spots correctly</t>
+  </si>
+  <si>
+    <t>CheckAvailableSpots_FullyBooked</t>
+  </si>
+  <si>
+    <t>Open "Availablity" screen
+Select park : Banias Nature Reserve
+Select date &amp; time : 07/04/2026, 14:00</t>
+  </si>
+  <si>
+    <t>The system displays "Fully Booked"</t>
+  </si>
+  <si>
+    <t>Banias Nature Reserve is fully booked  for 07/04/2026 at 14:00</t>
+  </si>
+  <si>
+    <t>checking display when park is fully booked</t>
+  </si>
+  <si>
+    <t>CheckAvailableSpots_PartialSpace</t>
+  </si>
+  <si>
+    <t>Open booking screen
+Select park : Banias Nature Reserve
+Select date &amp; time : 08/04/2026, 10:00
+Enter number of visitors: 10
+Click "Book visit"</t>
+  </si>
+  <si>
+    <t>The system displays a warning message: "Only 5 spots left for this date &amp; time."</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banias Nature Reserve has only 5 spots available for 08/04/2026, 10:00 </t>
+  </si>
+  <si>
+    <t>requesting more spots than currently available</t>
+  </si>
+  <si>
+    <t>ReportExit_Successful</t>
+  </si>
+  <si>
+    <t>Open "Occupancy Management" screen
+Enter number of exiting visitors: 4
+Click "Report Exit"</t>
+  </si>
+  <si>
+    <t>The system decreases the current park occupancy by 4
+A success message is displayed</t>
+  </si>
+  <si>
+    <t>Employee is logged in.
+Current park occupancy is at least 4</t>
+  </si>
+  <si>
+    <t>standard manual exit report.</t>
+  </si>
+  <si>
+    <t>ReportExit_ByGroupLeadID</t>
+  </si>
+  <si>
+    <t>Open "Occupancy Management" screen
+Click "Group Exit"
+Enter booking lead's ID number
+Click "Report Exit"</t>
+  </si>
+  <si>
+    <t>System updates the status of the entire group to "Exited".
+Park occupancy decreases by the number of visitors in that booking</t>
+  </si>
+  <si>
+    <t>Employee is logged in.
+a group associated with that ID is currently marked as "Inside Park".</t>
+  </si>
+  <si>
+    <t>Entering the group leader's ID on exit marks the whole group is exited and decreases the total number of visitors accordingly</t>
+  </si>
+  <si>
+    <t>Check the available spots in the park
+Perform exit report
+Check the available spots in the park (again)</t>
+  </si>
+  <si>
+    <t>The system accurately displays the number of visitors before the exit, and then after the group exits (e.g. 4 people) the number is decreased by 4.</t>
+  </si>
+  <si>
+    <t>Employee is logged in.
+Current park occupancy is at least 4 and a group of size 4 exists in the park</t>
+  </si>
+  <si>
+    <t>Verify system correctly calculates occupancy in real-time.</t>
+  </si>
+  <si>
+    <t>GenerateBill_PrebookedFamily</t>
+  </si>
+  <si>
+    <t>Open "Entrance Management" screen
+Click "Individual/Family visit" button
+Enter reservation ID
+Click "Generate Bill" button</t>
+  </si>
+  <si>
+    <t>System generates a bill with 15% discount.</t>
+  </si>
+  <si>
+    <t>A group associated with the 
+ID in the reservation exists</t>
+  </si>
+  <si>
+    <t>Pricing type 1</t>
+  </si>
+  <si>
+    <t>GenerateBill_CasualVisit</t>
+  </si>
+  <si>
+    <t>Open "Entrance Management" screen
+Click "Casual visit" button
+Select "Indiviual / Familiy"
+Enter number of visitors
+Click "Generate Bill" button</t>
+  </si>
+  <si>
+    <t>System generates bill at full price
+(no discount)</t>
+  </si>
+  <si>
+    <t>Availalble space for number of visitors</t>
+  </si>
+  <si>
+    <t>Pricing type 2</t>
+  </si>
+  <si>
+    <t>GenerateBill_PrebookedGroup_FrontalPay</t>
+  </si>
+  <si>
+    <t>Open "Entrance Management" screen
+Click "Group visit" button
+Enter reservation ID
+Click "Generate Bill" button</t>
+  </si>
+  <si>
+    <t>System generates a bill with 25% discount.
+Guide is charged 0. (Bill doesn’t include guide)</t>
+  </si>
+  <si>
+    <t>Pricing type 3 - frontal pay</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">GenerateBill_PrebookedGroup_Prepay 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(לא בטוח לגבי זה)</t>
+    </r>
+  </si>
+  <si>
+    <t>Open booking screen
+Enter visitor ID
+Select park: Banias Nature Reserve
+Select date and time: 16/04/2026 11:00
+Enter number of visitors: 12
+Enter e-mail: guide@gmail.com
+Click "book visit" button
+(?) Click "Prepay" button (?)</t>
+  </si>
+  <si>
+    <t>System generates a bill with 37% discount.
+Guide is charged 0. (Bill doesn’t include guide)</t>
+  </si>
+  <si>
+    <t>The group guide is registered in the system.
+Banias Nature Reserve has available capacity for 12 visitors on 16/04/2026 at 11:00.</t>
+  </si>
+  <si>
+    <t>Pricing type 3 - prepay</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">GenerateBill_CasualGroup
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>לא סגור אם זה אפשרי בכלל בסיפור אבל נראלי שכן כי לא כתוב שלא (או ספספתי)</t>
+    </r>
+  </si>
+  <si>
+    <t>Open "Entrance Management" screen
+Click "Casual visit" button
+Select "Organized Group"
+Enter number of visitors
+Click "Generate Bill" button</t>
+  </si>
+  <si>
+    <t>System generates a bill with a discount of 10%.
+Guide is charged normally. (Bill includes guide)</t>
+  </si>
+  <si>
+    <t>The group guide is registered in the system.
+Available space for number of visitors</t>
+  </si>
+  <si>
+    <t>Pricing type 4</t>
+  </si>
+  <si>
+    <t>GenerateBill_Subscriber_CasualVisit</t>
+  </si>
+  <si>
+    <t>Open "Entrance Management" screen
+Click "Member visit" button
+Enter Subscriber ID
+Click "Identify visitor"
+Enter number of visitors
+Click "Generate Bill" button</t>
+  </si>
+  <si>
+    <t>System generates a bill applying 10% subscriber discount to the full regular price.</t>
+  </si>
+  <si>
+    <t>Visitor has an active subscriber status.
+No prior reservation exists.
+Park has available space.</t>
+  </si>
+  <si>
+    <t>Pricing type 5 - casual visit</t>
+  </si>
+  <si>
+    <t>GenerateBill_Subscriber_Prebooked</t>
+  </si>
+  <si>
+    <t>Open "Entrance Management" screen
+Click "Member visit" button
+Enter Subscriber ID
+Click "Identify visitor"
+System presents booking
+Click "Generate Bill" button</t>
+  </si>
+  <si>
+    <t>System generates bill applying multiple discounts : 15% (prebook) + 10% (subscriber).
+In total 25% discount</t>
+  </si>
+  <si>
+    <t>Visitor has an active subscriber status.
+A valid reservations for that visitor exists</t>
+  </si>
+  <si>
+    <t>Pricint type 5 - booked visit</t>
+  </si>
+  <si>
+    <t>GenerateReport_Visitor_Successful</t>
+  </si>
+  <si>
+    <t>Open "Reports" screen
+Select "Visitor Report".
+Select date : 04/2026
+Click "Generate Report"</t>
+  </si>
+  <si>
+    <t>System generates a report detailing entry times and stay durations,
+ segmented by individuals and organized groups.
+The report is presented as a visual/graphical representation.</t>
+  </si>
+  <si>
+    <t>User is logged in as a Department Manager.
+Database contains visitor entry/exit records for the selected month.</t>
+  </si>
+  <si>
+    <t>Generate visitor report for a 
+period with existing visitor activity.</t>
+  </si>
+  <si>
+    <t>GenerateReport_Visitor_Unsuccessful</t>
+  </si>
+  <si>
+    <t>Open "Reports" screen
+Select "Visitor Report".
+Select date : 04/2027
+Click "Generate Report"</t>
+  </si>
+  <si>
+    <t>System displays message
+"No data available for selected period".</t>
+  </si>
+  <si>
+    <t>User is logged in as a Department Manager.
+Database contains no visitor entry/exit records for the selected month.</t>
+  </si>
+  <si>
+    <t>Generate visitor report for a 
+period with no existing visitor activity.</t>
+  </si>
+  <si>
+    <t>RecordEntryTime_UponCheckin</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Open "Entrance Management" screen
+Click "Individual/Family visit" button
+Enter reservation ID
+Click "Confirm Entry" button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Open visitor log or database record (?)</t>
+    </r>
+  </si>
+  <si>
+    <t>The system saves the exact time of the "Confirm Entry" action as the visitor's entry time.</t>
+  </si>
+  <si>
+    <t>Park employee is logged in.
+Visitor has a prepaid reservation.</t>
+  </si>
+  <si>
+    <t>Check if the system records the currect timestamp when a visitor enters</t>
+  </si>
+  <si>
+    <t>CalculateDuration_BasedOnEntryTime</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Open "Exit Management" screen
+Click "Individual/Family visit" button
+Enter reservation ID
+Click "Confirm Exit" button
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Open visitor log or database record (?)</t>
+    </r>
+  </si>
+  <si>
+    <t>The system correctly calculates the stay duration by subtracting the saved entry time from the current exit time.</t>
+  </si>
+  <si>
+    <t>Visitor is currently in the 
+park with previously recorded entry time</t>
+  </si>
+  <si>
+    <t>check if the system correctly caculates stay duration upon exit</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>(?)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> CheckOccupancy_AfterExit</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1055,14 +1463,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1082,7 +1490,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1090,9 +1498,32 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1207,7 +1638,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1246,13 +1677,26 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1276,7 +1720,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ערכת נושא של Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -1573,11 +2017,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABE2F884-F2EF-4287-AC3D-5537D5275C3C}">
   <dimension ref="A1:C83"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5" customWidth="1"/>
-    <col min="2" max="2" width="88.09765625" customWidth="1"/>
-    <col min="3" max="3" width="5.19921875" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" customWidth="1"/>
+    <col min="2" max="2" width="88.140625" customWidth="1"/>
+    <col min="3" max="3" width="5.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="16" customFormat="1" ht="93.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1585,7 +2029,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="121.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1618,7 +2062,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1761,7 +2205,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -2487,22 +2931,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A028A801-0122-4DDE-8D73-57AF100E1B01}">
-  <dimension ref="A1:Z42"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Z62"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="79.69921875" customWidth="1"/>
-    <col min="2" max="2" width="36.8984375" customWidth="1"/>
-    <col min="3" max="3" width="39.19921875" customWidth="1"/>
-    <col min="4" max="4" width="24.69921875" customWidth="1"/>
+    <col min="1" max="1" width="79.7109375" customWidth="1"/>
+    <col min="2" max="2" width="36.85546875" customWidth="1"/>
+    <col min="3" max="3" width="39.140625" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="16" customFormat="1" ht="88.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="16" customFormat="1" ht="88.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2519,7 +2963,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="55.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" s="2" customFormat="1" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>90</v>
       </c>
@@ -2553,7 +2997,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="83.4" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>100</v>
       </c>
@@ -2570,7 +3014,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="83.4" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>105</v>
       </c>
@@ -2587,7 +3031,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="97.2" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>107</v>
       </c>
@@ -2604,7 +3048,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="55.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>109</v>
       </c>
@@ -2621,7 +3065,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="124.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>114</v>
       </c>
@@ -2638,7 +3082,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="124.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>119</v>
       </c>
@@ -2655,7 +3099,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="124.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>121</v>
       </c>
@@ -2672,7 +3116,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="124.8" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>126</v>
       </c>
@@ -2689,7 +3133,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="138.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>131</v>
       </c>
@@ -2706,7 +3150,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>136</v>
       </c>
@@ -2723,7 +3167,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
         <v>141</v>
       </c>
@@ -2740,7 +3184,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="83.4" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>145</v>
       </c>
@@ -2757,7 +3201,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="207.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" ht="195.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
         <v>150</v>
       </c>
@@ -2774,7 +3218,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="207.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" ht="195.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>155</v>
       </c>
@@ -2791,7 +3235,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="88.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" ht="88.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
         <v>159</v>
       </c>
@@ -2808,7 +3252,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="90.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" ht="95.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
         <v>164</v>
       </c>
@@ -2825,7 +3269,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="157.80000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" ht="157.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
         <v>168</v>
       </c>
@@ -2842,7 +3286,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="157.80000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" ht="157.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
         <v>173</v>
       </c>
@@ -2859,7 +3303,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" ht="95.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>177</v>
       </c>
@@ -2876,7 +3320,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="135.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" ht="111" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>181</v>
       </c>
@@ -2893,7 +3337,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="135.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" ht="111" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
         <v>185</v>
       </c>
@@ -2910,7 +3354,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>189</v>
       </c>
@@ -2927,7 +3371,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
         <v>194</v>
       </c>
@@ -2944,7 +3388,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" ht="111" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>198</v>
       </c>
@@ -2961,7 +3405,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="135.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" ht="111" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>203</v>
       </c>
@@ -2978,7 +3422,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" ht="95.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>206</v>
       </c>
@@ -2995,7 +3439,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>210</v>
       </c>
@@ -3012,7 +3456,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="136.80000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" ht="136.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
         <v>215</v>
       </c>
@@ -3029,7 +3473,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="33" spans="1:26" ht="131.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:26" ht="131.44999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
         <v>219</v>
       </c>
@@ -3046,7 +3490,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="34" spans="1:26" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:26" ht="111" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>220</v>
       </c>
@@ -3063,7 +3507,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="35" spans="1:26" ht="120.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:26" ht="111" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>224</v>
       </c>
@@ -3080,7 +3524,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="36" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:26" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
         <v>228</v>
       </c>
@@ -3097,7 +3541,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="37" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:26" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="s">
         <v>233</v>
       </c>
@@ -3114,7 +3558,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="38" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:26" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="s">
         <v>233</v>
       </c>
@@ -3131,7 +3575,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="39" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:26" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
         <v>236</v>
       </c>
@@ -3169,7 +3613,7 @@
       <c r="Y39" s="13"/>
       <c r="Z39" s="13"/>
     </row>
-    <row r="40" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:26" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
         <v>241</v>
       </c>
@@ -3207,7 +3651,7 @@
       <c r="Y40" s="13"/>
       <c r="Z40" s="13"/>
     </row>
-    <row r="41" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:26" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="11" t="s">
         <v>246</v>
       </c>
@@ -3245,7 +3689,7 @@
       <c r="Y41" s="13"/>
       <c r="Z41" s="13"/>
     </row>
-    <row r="42" spans="1:26" ht="169.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:26" ht="169.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="11" t="s">
         <v>250</v>
       </c>
@@ -3283,6 +3727,315 @@
       <c r="Y42" s="13"/>
       <c r="Z42" s="13"/>
     </row>
+    <row r="43" spans="1:26" ht="95.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="17" t="s">
+        <v>260</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>261</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="D43" s="18" t="s">
+        <v>263</v>
+      </c>
+      <c r="E43" s="18" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="44" spans="1:26" ht="79.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="18" t="s">
+        <v>265</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>266</v>
+      </c>
+      <c r="C44" s="18" t="s">
+        <v>267</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="E44" s="18" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="45" spans="1:26" ht="111" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="C45" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="D45" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="E45" s="18" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="46" spans="1:26" ht="79.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="19" t="s">
+        <v>275</v>
+      </c>
+      <c r="B46" s="20" t="s">
+        <v>276</v>
+      </c>
+      <c r="C46" s="20" t="s">
+        <v>277</v>
+      </c>
+      <c r="D46" s="20" t="s">
+        <v>278</v>
+      </c>
+      <c r="E46" s="20" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="47" spans="1:26" ht="111" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="19" t="s">
+        <v>280</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="D47" s="20" t="s">
+        <v>283</v>
+      </c>
+      <c r="E47" s="20" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="48" spans="1:26" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A48" s="19" t="s">
+        <v>343</v>
+      </c>
+      <c r="B48" s="20" t="s">
+        <v>285</v>
+      </c>
+      <c r="C48" s="20" t="s">
+        <v>286</v>
+      </c>
+      <c r="D48" s="20" t="s">
+        <v>287</v>
+      </c>
+      <c r="E48" s="20" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+    </row>
+    <row r="50" spans="1:5" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="19" t="s">
+        <v>289</v>
+      </c>
+      <c r="B50" s="20" t="s">
+        <v>290</v>
+      </c>
+      <c r="C50" s="19" t="s">
+        <v>291</v>
+      </c>
+      <c r="D50" s="20" t="s">
+        <v>292</v>
+      </c>
+      <c r="E50" s="19" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A51" s="19" t="s">
+        <v>294</v>
+      </c>
+      <c r="B51" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C51" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="D51" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A52" s="19" t="s">
+        <v>299</v>
+      </c>
+      <c r="B52" s="20" t="s">
+        <v>300</v>
+      </c>
+      <c r="C52" s="20" t="s">
+        <v>301</v>
+      </c>
+      <c r="D52" s="20" t="s">
+        <v>292</v>
+      </c>
+      <c r="E52" s="19" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="157.5" x14ac:dyDescent="0.25">
+      <c r="A53" s="20" t="s">
+        <v>303</v>
+      </c>
+      <c r="B53" s="20" t="s">
+        <v>304</v>
+      </c>
+      <c r="C53" s="20" t="s">
+        <v>305</v>
+      </c>
+      <c r="D53" s="20" t="s">
+        <v>306</v>
+      </c>
+      <c r="E53" s="19" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A54" s="20" t="s">
+        <v>308</v>
+      </c>
+      <c r="B54" s="20" t="s">
+        <v>309</v>
+      </c>
+      <c r="C54" s="20" t="s">
+        <v>310</v>
+      </c>
+      <c r="D54" s="20" t="s">
+        <v>311</v>
+      </c>
+      <c r="E54" s="19" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A55" s="19" t="s">
+        <v>313</v>
+      </c>
+      <c r="B55" s="20" t="s">
+        <v>314</v>
+      </c>
+      <c r="C55" s="20" t="s">
+        <v>315</v>
+      </c>
+      <c r="D55" s="20" t="s">
+        <v>316</v>
+      </c>
+      <c r="E55" s="19" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A56" s="19" t="s">
+        <v>318</v>
+      </c>
+      <c r="B56" s="20" t="s">
+        <v>319</v>
+      </c>
+      <c r="C56" s="20" t="s">
+        <v>320</v>
+      </c>
+      <c r="D56" s="20" t="s">
+        <v>321</v>
+      </c>
+      <c r="E56" s="19" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A57" s="19"/>
+      <c r="B57" s="19"/>
+      <c r="C57" s="19"/>
+      <c r="D57" s="19"/>
+      <c r="E57" s="19"/>
+    </row>
+    <row r="58" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A58" s="19" t="s">
+        <v>323</v>
+      </c>
+      <c r="B58" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="C58" s="20" t="s">
+        <v>325</v>
+      </c>
+      <c r="D58" s="20" t="s">
+        <v>326</v>
+      </c>
+      <c r="E58" s="20" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A59" s="19" t="s">
+        <v>328</v>
+      </c>
+      <c r="B59" s="20" t="s">
+        <v>329</v>
+      </c>
+      <c r="C59" s="20" t="s">
+        <v>330</v>
+      </c>
+      <c r="D59" s="20" t="s">
+        <v>331</v>
+      </c>
+      <c r="E59" s="20" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A60" s="21"/>
+      <c r="B60" s="21"/>
+      <c r="C60" s="21"/>
+      <c r="D60" s="21"/>
+      <c r="E60" s="21"/>
+    </row>
+    <row r="61" spans="1:5" ht="126" x14ac:dyDescent="0.25">
+      <c r="A61" s="19" t="s">
+        <v>333</v>
+      </c>
+      <c r="B61" s="20" t="s">
+        <v>334</v>
+      </c>
+      <c r="C61" s="20" t="s">
+        <v>335</v>
+      </c>
+      <c r="D61" s="20" t="s">
+        <v>336</v>
+      </c>
+      <c r="E61" s="20" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="126" x14ac:dyDescent="0.25">
+      <c r="A62" s="19" t="s">
+        <v>338</v>
+      </c>
+      <c r="B62" s="20" t="s">
+        <v>339</v>
+      </c>
+      <c r="C62" s="20" t="s">
+        <v>340</v>
+      </c>
+      <c r="D62" s="20" t="s">
+        <v>341</v>
+      </c>
+      <c r="E62" s="20" t="s">
+        <v>342</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:XFD1"/>

</xml_diff>